<commit_message>
model part of https://github.com/pydna-group/pydna/issues/435
</commit_message>
<xml_diff>
--- a/project/excel/opencloning_linkml.xlsx
+++ b/project/excel/opencloning_linkml.xlsx
@@ -49,13 +49,15 @@
     <sheet name="CRISPRSource" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="OligoHybridizationSource" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="PolymeraseExtensionSource" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="CloningStrategy" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="AnnotationReport" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="PlannotateAnnotationReport" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="AnnotationSource" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="ReverseComplementSource" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="AssociatedFile" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="SequencingFile" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="Recombinase" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="RecombinaseSource" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="CloningStrategy" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="AnnotationReport" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="PlannotateAnnotationReport" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="AnnotationSource" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="ReverseComplementSource" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="AssociatedFile" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="SequencingFile" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2243,12 +2245,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>site1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>site2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>site1_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>site2_name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>recombinases</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>reverse_reaction</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>circular</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>output_name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>database_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>sequences</t>
         </is>
       </c>
@@ -2293,7 +2392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2314,7 +2413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2405,7 +2504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2466,7 +2565,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2507,7 +2606,48 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>database_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2548,7 +2688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2594,7 +2734,90 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cut_watson</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>overhang</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>restriction_enzyme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>cut_watson</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>overhang</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2606,130 +2829,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>database_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sequence</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sequence</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>cut_watson</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>overhang</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>restriction_enzyme</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>cut_watson</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>overhang</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t>database_id</t>
         </is>
       </c>

</xml_diff>

<commit_message>
remove reverse from source
</commit_message>
<xml_diff>
--- a/project/excel/opencloning_linkml.xlsx
+++ b/project/excel/opencloning_linkml.xlsx
@@ -2286,7 +2286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2297,35 +2297,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>reverse_reaction</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>circular</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>output_name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>database_id</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>output_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>database_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>input</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>id</t>
         </is>

</xml_diff>